<commit_message>
Modificaciones de las plantillas
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="oficio" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -39,13 +39,6 @@
     <font>
       <name val="Times New Roman"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Times New Roman"/>
@@ -99,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -108,13 +101,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -192,7 +184,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -383,44 +375,46 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <dimension ref="A1:AL2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="15.42578125" customWidth="1" min="7" max="8"/>
-    <col width="12.5703125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="15.42578125" customWidth="1" style="10" min="7" max="7"/>
+    <col width="17.85546875" customWidth="1" style="10" min="8" max="8"/>
+    <col width="12.5703125" bestFit="1" customWidth="1" style="10" min="9" max="9"/>
     <col width="14" bestFit="1" customWidth="1" style="1" min="10" max="10"/>
-    <col width="35.28515625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="16.42578125" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="11.85546875" bestFit="1" customWidth="1" min="13" max="13"/>
-    <col width="13.140625" bestFit="1" customWidth="1" min="14" max="14"/>
-    <col width="15.42578125" bestFit="1" customWidth="1" min="15" max="15"/>
-    <col width="14.5703125" bestFit="1" customWidth="1" min="16" max="16"/>
-    <col width="31" bestFit="1" customWidth="1" min="17" max="17"/>
-    <col width="20.85546875" customWidth="1" min="18" max="19"/>
-    <col width="15.85546875" bestFit="1" customWidth="1" min="20" max="20"/>
-    <col width="14.85546875" bestFit="1" customWidth="1" min="21" max="21"/>
-    <col width="14.42578125" bestFit="1" customWidth="1" min="22" max="22"/>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="23" max="23"/>
-    <col width="13" bestFit="1" customWidth="1" min="24" max="24"/>
-    <col width="20" bestFit="1" customWidth="1" min="25" max="25"/>
-    <col width="19.42578125" bestFit="1" customWidth="1" min="26" max="26"/>
-    <col width="22.140625" bestFit="1" customWidth="1" min="27" max="27"/>
-    <col width="22.42578125" bestFit="1" customWidth="1" min="28" max="28"/>
-    <col width="22.42578125" customWidth="1" min="29" max="32"/>
-    <col width="25.40234375" bestFit="1" customWidth="1" min="33" max="33"/>
-    <col width="25.40234375" customWidth="1" min="34" max="37"/>
+    <col width="35.28515625" bestFit="1" customWidth="1" style="10" min="11" max="11"/>
+    <col width="16.42578125" bestFit="1" customWidth="1" style="10" min="12" max="12"/>
+    <col width="11.85546875" bestFit="1" customWidth="1" style="10" min="13" max="13"/>
+    <col width="13.140625" bestFit="1" customWidth="1" style="10" min="14" max="14"/>
+    <col width="15.42578125" bestFit="1" customWidth="1" style="10" min="15" max="15"/>
+    <col width="14.5703125" bestFit="1" customWidth="1" style="10" min="16" max="16"/>
+    <col width="31" bestFit="1" customWidth="1" style="10" min="17" max="17"/>
+    <col width="20.85546875" customWidth="1" style="10" min="18" max="19"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" style="10" min="20" max="20"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" style="10" min="21" max="21"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" style="10" min="22" max="22"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="23" max="23"/>
+    <col width="13" bestFit="1" customWidth="1" style="10" min="24" max="24"/>
+    <col width="20" bestFit="1" customWidth="1" style="10" min="25" max="25"/>
+    <col width="19.42578125" bestFit="1" customWidth="1" style="10" min="26" max="26"/>
+    <col width="22.140625" bestFit="1" customWidth="1" style="10" min="27" max="27"/>
+    <col width="22.42578125" bestFit="1" customWidth="1" style="10" min="28" max="28"/>
+    <col width="22.42578125" customWidth="1" style="10" min="29" max="32"/>
+    <col width="25.42578125" bestFit="1" customWidth="1" style="10" min="33" max="33"/>
+    <col width="25.42578125" customWidth="1" style="10" min="34" max="37"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1" s="10">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>registro</t>
@@ -613,8 +607,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
-        <v>49</v>
+      <c r="A2" t="n">
+        <v>56</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
@@ -631,70 +625,68 @@
           <t xml:space="preserve"> David</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 12/03/2026</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="E2" s="9" t="n">
+        <v>46359</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>11:00 a.m.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Oficina Judicial</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Licda. Aivys Castillo</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>6216 (843-26)</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>202500001193</v>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Contra La Libertad e Integridad Sexual</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Actos Libidinosos</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  David</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Investigación</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="n">
+        <v>46129</v>
+      </c>
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>10:00 a.m.</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Oficina Judicial</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Licda. Aivys Castillo</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>6315 (840-26)</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="n">
-        <v>202400008107</v>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Contra La Libertad e Integridad Sexual</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>Violación</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  David</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Investigación</t>
-        </is>
-      </c>
-      <c r="O2" s="7" t="n">
-        <v>46238</v>
-      </c>
-      <c r="P2" s="7" t="inlineStr">
-        <is>
-          <t>9:00 a.m.</t>
-        </is>
-      </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve"> Anticipo Jurisdiccional de Prueba</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
-        <is>
-          <t>Barbara Delgado</t>
+      <c r="R2" s="11" t="inlineStr">
+        <is>
+          <t>Yinel Saldaña</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
@@ -702,9 +694,9 @@
           <t>Enrique Jimenez</t>
         </is>
       </c>
-      <c r="T2" s="5" t="inlineStr">
-        <is>
-          <t>R.Y.P.M.</t>
+      <c r="T2" s="11" t="inlineStr">
+        <is>
+          <t>M.V.DG.M.</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
@@ -712,19 +704,19 @@
           <t>Femenino</t>
         </is>
       </c>
-      <c r="V2" s="5" t="inlineStr">
-        <is>
-          <t>4-854-283</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="inlineStr">
-        <is>
-          <t>20/03/2010</t>
-        </is>
-      </c>
-      <c r="X2" s="5" t="inlineStr">
-        <is>
-          <t>10 años</t>
+      <c r="V2" s="11" t="inlineStr">
+        <is>
+          <t>4-894-1660</t>
+        </is>
+      </c>
+      <c r="W2" s="11" t="inlineStr">
+        <is>
+          <t>24/05/2019</t>
+        </is>
+      </c>
+      <c r="X2" s="11" t="inlineStr">
+        <is>
+          <t>06 años</t>
         </is>
       </c>
       <c r="Y2" s="5" t="inlineStr">
@@ -732,270 +724,86 @@
           <t>Panameña</t>
         </is>
       </c>
-      <c r="Z2" s="5" t="inlineStr">
-        <is>
-          <t>Luis Eduardo Olmo</t>
-        </is>
-      </c>
-      <c r="AA2" s="5" t="inlineStr">
-        <is>
-          <t>24 años, Masculino.</t>
-        </is>
-      </c>
-      <c r="AB2" s="5" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
-      <c r="AC2" s="5" t="inlineStr">
-        <is>
-          <t>Coordinadora</t>
-        </is>
-      </c>
-      <c r="AD2" s="5" t="inlineStr">
-        <is>
-          <t>operador</t>
-        </is>
-      </c>
-      <c r="AE2" s="5" t="inlineStr">
-        <is>
-          <t>16 de abril</t>
-        </is>
-      </c>
-      <c r="AF2" s="5" t="n">
-        <v>1333</v>
-      </c>
-      <c r="AG2" s="5" t="inlineStr">
-        <is>
-          <t>Aivys Castillo</t>
-        </is>
-      </c>
-      <c r="AH2" s="5" t="inlineStr">
+      <c r="Z2" s="11" t="inlineStr">
+        <is>
+          <t>Roderick Jahir Pitti De Gracia</t>
+        </is>
+      </c>
+      <c r="AA2" s="11" t="inlineStr">
+        <is>
+          <t>27 años, Masculino</t>
+        </is>
+      </c>
+      <c r="AB2" s="11" t="inlineStr">
+        <is>
+          <t>Padrastro</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Ann Lynn Rios</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Enrique Jimenez</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>17 de abril</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>AIVYS CASTILLO</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>CASTILLO</t>
         </is>
       </c>
-      <c r="AI2" s="5" t="inlineStr">
-        <is>
-          <t>Tres (3)</t>
-        </is>
-      </c>
-      <c r="AJ2" s="5" t="inlineStr">
-        <is>
-          <t>Fiscalia, Defensa</t>
-        </is>
-      </c>
-      <c r="AK2" s="5" t="n">
-        <v>4569</v>
-      </c>
-      <c r="AL2" s="5" t="inlineStr">
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Cuatro (4)</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Fiscalia, Defensa y Querella</t>
+        </is>
+      </c>
+      <c r="AK2" t="n">
+        <v>6216</v>
+      </c>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" t="n">
-        <v>100</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Chiriquí</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> David</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> David</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>46188</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>11:00 a.m.</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Oficina Judicial</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Licda. Aivys Castillo</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>6000 (800-26)</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>202500000001</v>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Contra La Libertad e Integridad Sexual</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>Violación</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  David</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Investigación</t>
-        </is>
-      </c>
-      <c r="O3" s="9" t="n">
-        <v>46189</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2:00 p.m.</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Anticipo Jurisdiccional de Prueba</t>
-        </is>
-      </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>Barbara Delgado</t>
-        </is>
-      </c>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>Enrique Jimenez</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>A.A.A.A.</t>
-        </is>
-      </c>
-      <c r="U3" s="5" t="inlineStr">
-        <is>
-          <t>Femenino</t>
-        </is>
-      </c>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>4-854-283</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
-        <is>
-          <t>20/03/2010</t>
-        </is>
-      </c>
-      <c r="X3" s="5" t="inlineStr">
-        <is>
-          <t>10 años</t>
-        </is>
-      </c>
-      <c r="Y3" s="5" t="inlineStr">
-        <is>
-          <t>Panameña</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>HOLA hola</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>25 anos, Masculino</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Padre</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Ann Lynn Rios</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>Enrique Jimenez</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20 de abril </t>
-        </is>
-      </c>
-      <c r="AF3" t="n">
-        <v>2587</v>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>YASLEL VIL</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>VIL</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>Cuatro (4)</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>Fiscalia, Defensa y Querella</t>
-        </is>
-      </c>
-      <c r="AK3" t="n">
-        <v>1111</v>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="O4" s="10" t="n"/>
-    </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="4294967294" verticalDpi="4294967294" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="4294967294" verticalDpi="4294967294"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="19.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="19.28515625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
+    <col width="19.85546875" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="19.28515625" bestFit="1" customWidth="1" style="10" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1255,7 +1063,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>coodinadora</t>
         </is>
@@ -1267,7 +1075,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>tecnico_operador</t>
         </is>
@@ -1279,23 +1087,22 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="23.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
+    <col width="23.42578125" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1635,7 +1442,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>coodinadora</t>
         </is>
@@ -1647,7 +1454,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>tecnico_operador</t>
         </is>
@@ -1659,23 +1466,22 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="23.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
+    <col width="23.42578125" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2015,7 +1821,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>coodinadora</t>
         </is>
@@ -2027,7 +1833,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>tecnico_operador</t>
         </is>
@@ -2039,22 +1845,21 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A15:A26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="18.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18.28515625" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="15">
@@ -2134,16 +1939,15 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
+    <row r="26" ht="16.5" customHeight="1" s="10">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>victima</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="4294967294" verticalDpi="4294967294" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="4294967294" verticalDpi="4294967294"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Otras Modificaciones de las plantillas
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -22,9 +22,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -92,21 +99,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -607,7 +615,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="12" t="n">
         <v>56</v>
       </c>
       <c r="B2" s="5" t="inlineStr">

</xml_diff>

<commit_message>
agrega git ignore a output
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>11:00 a.m.</t>
+          <t>09:07 a.m.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="T2" s="11" t="inlineStr">
         <is>
-          <t>M.V.DG.M.</t>
+          <t>M.V.D.M.</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>Ann Lynn Rios</t>
+          <t>Ann Lynn Rios Rios</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -761,9 +761,6 @@
         <is>
           <t>17 de abril</t>
         </is>
-      </c>
-      <c r="AF2" t="n">
-        <v>1000</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cambio de nombre de carpeta de salida
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -61,7 +61,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -95,11 +95,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +124,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,36 +405,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL2"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="15.42578125" customWidth="1" style="10" min="7" max="7"/>
-    <col width="17.85546875" customWidth="1" style="10" min="8" max="8"/>
-    <col width="12.5703125" bestFit="1" customWidth="1" style="10" min="9" max="9"/>
+    <col width="15.42578125" customWidth="1" style="15" min="7" max="7"/>
+    <col width="17.85546875" customWidth="1" style="15" min="8" max="8"/>
+    <col width="12.5703125" bestFit="1" customWidth="1" style="15" min="9" max="9"/>
     <col width="14" bestFit="1" customWidth="1" style="1" min="10" max="10"/>
-    <col width="35.28515625" bestFit="1" customWidth="1" style="10" min="11" max="11"/>
-    <col width="16.42578125" bestFit="1" customWidth="1" style="10" min="12" max="12"/>
-    <col width="11.85546875" bestFit="1" customWidth="1" style="10" min="13" max="13"/>
-    <col width="13.140625" bestFit="1" customWidth="1" style="10" min="14" max="14"/>
-    <col width="15.42578125" bestFit="1" customWidth="1" style="10" min="15" max="15"/>
-    <col width="14.5703125" bestFit="1" customWidth="1" style="10" min="16" max="16"/>
-    <col width="31" bestFit="1" customWidth="1" style="10" min="17" max="17"/>
-    <col width="20.85546875" customWidth="1" style="10" min="18" max="19"/>
-    <col width="15.85546875" bestFit="1" customWidth="1" style="10" min="20" max="20"/>
-    <col width="14.85546875" bestFit="1" customWidth="1" style="10" min="21" max="21"/>
-    <col width="14.42578125" bestFit="1" customWidth="1" style="10" min="22" max="22"/>
-    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="23" max="23"/>
-    <col width="13" bestFit="1" customWidth="1" style="10" min="24" max="24"/>
-    <col width="20" bestFit="1" customWidth="1" style="10" min="25" max="25"/>
-    <col width="19.42578125" bestFit="1" customWidth="1" style="10" min="26" max="26"/>
-    <col width="22.140625" bestFit="1" customWidth="1" style="10" min="27" max="27"/>
-    <col width="22.42578125" bestFit="1" customWidth="1" style="10" min="28" max="28"/>
-    <col width="22.42578125" customWidth="1" style="10" min="29" max="32"/>
-    <col width="25.42578125" bestFit="1" customWidth="1" style="10" min="33" max="33"/>
-    <col width="25.42578125" customWidth="1" style="10" min="34" max="37"/>
+    <col width="35.28515625" bestFit="1" customWidth="1" style="15" min="11" max="11"/>
+    <col width="16.42578125" bestFit="1" customWidth="1" style="15" min="12" max="12"/>
+    <col width="11.85546875" bestFit="1" customWidth="1" style="15" min="13" max="13"/>
+    <col width="13.140625" bestFit="1" customWidth="1" style="15" min="14" max="14"/>
+    <col width="15.42578125" bestFit="1" customWidth="1" style="15" min="15" max="15"/>
+    <col width="14.5703125" bestFit="1" customWidth="1" style="15" min="16" max="16"/>
+    <col width="31" bestFit="1" customWidth="1" style="15" min="17" max="17"/>
+    <col width="20.85546875" customWidth="1" style="15" min="18" max="19"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" style="15" min="20" max="20"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" style="15" min="21" max="21"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" style="15" min="22" max="22"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="15" min="23" max="23"/>
+    <col width="13" bestFit="1" customWidth="1" style="15" min="24" max="24"/>
+    <col width="20" bestFit="1" customWidth="1" style="15" min="25" max="25"/>
+    <col width="19.42578125" bestFit="1" customWidth="1" style="15" min="26" max="26"/>
+    <col width="22.140625" bestFit="1" customWidth="1" style="15" min="27" max="27"/>
+    <col width="22.42578125" bestFit="1" customWidth="1" style="15" min="28" max="28"/>
+    <col width="22.42578125" customWidth="1" style="15" min="29" max="32"/>
+    <col width="25.42578125" bestFit="1" customWidth="1" style="15" min="33" max="33"/>
+    <col width="25.42578125" customWidth="1" style="15" min="34" max="37"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="10">
+    <row r="1" ht="15.75" customHeight="1" s="15">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>registro</t>
@@ -682,7 +694,7 @@
       <c r="O2" s="6" t="n">
         <v>46129</v>
       </c>
-      <c r="P2" s="11" t="inlineStr">
+      <c r="P2" s="14" t="inlineStr">
         <is>
           <t>10:00 a.m.</t>
         </is>
@@ -692,7 +704,7 @@
           <t xml:space="preserve"> Anticipo Jurisdiccional de Prueba</t>
         </is>
       </c>
-      <c r="R2" s="11" t="inlineStr">
+      <c r="R2" s="14" t="inlineStr">
         <is>
           <t>Yinel Saldaña</t>
         </is>
@@ -702,29 +714,29 @@
           <t>Enrique Jimenez</t>
         </is>
       </c>
-      <c r="T2" s="11" t="inlineStr">
-        <is>
-          <t>M.V.D.M.</t>
+      <c r="T2" s="14" t="inlineStr">
+        <is>
+          <t>M.V.D.M.  -  E.D.M.</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>Femenino</t>
-        </is>
-      </c>
-      <c r="V2" s="11" t="inlineStr">
-        <is>
-          <t>4-894-1660</t>
-        </is>
-      </c>
-      <c r="W2" s="11" t="inlineStr">
-        <is>
-          <t>24/05/2019</t>
-        </is>
-      </c>
-      <c r="X2" s="11" t="inlineStr">
-        <is>
-          <t>06 años</t>
+          <t>F - M</t>
+        </is>
+      </c>
+      <c r="V2" s="14" t="inlineStr">
+        <is>
+          <t>4-894-1660  -  4-906-1036</t>
+        </is>
+      </c>
+      <c r="W2" s="14" t="inlineStr">
+        <is>
+          <t>24/05/2019  /  10/12/2021</t>
+        </is>
+      </c>
+      <c r="X2" s="14" t="inlineStr">
+        <is>
+          <t>06 -  04 años</t>
         </is>
       </c>
       <c r="Y2" s="5" t="inlineStr">
@@ -732,17 +744,17 @@
           <t>Panameña</t>
         </is>
       </c>
-      <c r="Z2" s="11" t="inlineStr">
+      <c r="Z2" s="14" t="inlineStr">
         <is>
           <t>Roderick Jahir Pitti De Gracia</t>
         </is>
       </c>
-      <c r="AA2" s="11" t="inlineStr">
+      <c r="AA2" s="14" t="inlineStr">
         <is>
           <t>27 años, Masculino</t>
         </is>
       </c>
-      <c r="AB2" s="11" t="inlineStr">
+      <c r="AB2" s="14" t="inlineStr">
         <is>
           <t>Padrastro</t>
         </is>
@@ -786,6 +798,185 @@
         <v>6216</v>
       </c>
       <c r="AL2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Chiriquí</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> David</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> David</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>11:52 a.m.</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Oficina Judicial</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Licda. Aivys Castillo</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>7499 (951-26)</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>202500086032</v>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Contra La Libertad e Integridad Sexual</t>
+        </is>
+      </c>
+      <c r="L3" s="14" t="inlineStr">
+        <is>
+          <t>Violación</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  David</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Investigación</t>
+        </is>
+      </c>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="P3" s="14" t="inlineStr">
+        <is>
+          <t>2:00 a.m.</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Anticipo Jurisdiccional de Prueba</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Barbara Delgado</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Enrique Jimenez</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>A.L.G.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Femenino</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>4-861-684</t>
+        </is>
+      </c>
+      <c r="W3" s="9" t="n">
+        <v>40734</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>14 años</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>Panameña</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Adrian Alberto Ortega</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>21 años, Masculino</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Ann Lynn Rios Rios</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Enrique Jimenez</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>17 de abril</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>AIVYS CASTILLO</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>CASTILLO</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Cuatro (4)</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Fiscalia, Defensa y Querella</t>
+        </is>
+      </c>
+      <c r="AK3" t="n">
+        <v>7499</v>
+      </c>
+      <c r="AL3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
@@ -806,9 +997,9 @@
   <dimension ref="A2:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="19.85546875" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
-    <col width="19.28515625" bestFit="1" customWidth="1" style="10" min="8" max="8"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
+    <col width="19.85546875" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
+    <col width="19.28515625" bestFit="1" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1106,8 +1297,8 @@
   <dimension ref="A2:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="23.42578125" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
+    <col width="23.42578125" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1485,8 +1676,8 @@
   <dimension ref="A2:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="24.7109375" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="23.42578125" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="24.7109375" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
+    <col width="23.42578125" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1864,7 +2055,7 @@
   <dimension ref="A15:A26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="18.28515625" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
+    <col width="18.28515625" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="15">
@@ -1944,7 +2135,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="10">
+    <row r="26" ht="16.5" customHeight="1" s="15">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>victima</t>

</xml_diff>